<commit_message>
Update WorkLogs with latest changes
</commit_message>
<xml_diff>
--- a/WorkLogs.xlsx
+++ b/WorkLogs.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29721"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29803"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="80" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4DE3EFDC-88A0-414D-B732-37FEF1A37A72}"/>
+  <xr:revisionPtr revIDLastSave="84" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{26EFA01F-6EBC-4AA2-9D78-5C6191E1EBDB}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Khushi " sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="46">
   <si>
     <t>Date</t>
   </si>
@@ -277,6 +277,9 @@
   </si>
   <si>
     <t>complete proposal document</t>
+  </si>
+  <si>
+    <t xml:space="preserve">setup backend </t>
   </si>
 </sst>
 </file>
@@ -809,7 +812,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B04BA97-DE7E-4AE6-9FDB-13260294F106}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
@@ -938,6 +941,22 @@
         <v>44</v>
       </c>
     </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="1">
+        <v>46055</v>
+      </c>
+      <c r="B12">
+        <v>2</v>
+      </c>
+      <c r="C12" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="1">
+        <v>46114</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>